<commit_message>
chore(backlog): sync xlsx status for completed TSK
Mark TSK-193 (Wakil Direktur Utama Role in RBAC) as Done — covered by
TSK-003 RBAC engine + TSK-004 Permission Matrix (Wakil Direktur dapat
role terpisah dengan permission identik Direktur Utama, audit log persona
name eksplisit per NC-EX-005).

Current backlog state:
- Done: 68 task (432 story points)
- To Do: 135 task (~800 story points)
- 35% complete by SP

Next focus: M1.4 Payroll Foundation (TSK-046 s/d TSK-056 + TSK-194).
</commit_message>
<xml_diff>
--- a/IDEA_Task_Management.xlsx
+++ b/IDEA_Task_Management.xlsx
@@ -2089,7 +2089,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L203"/>
+  <dimension ref="A1:M206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2174,6 +2174,11 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>Completion Note</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="24" t="inlineStr">
@@ -2227,7 +2232,12 @@
       </c>
       <c r="L3" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>M1.1 — Single Login Portal</t>
         </is>
       </c>
     </row>
@@ -2287,7 +2297,12 @@
       </c>
       <c r="L4" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>M1.1 — JWT auth + refresh token rotation</t>
         </is>
       </c>
     </row>
@@ -2347,7 +2362,12 @@
       </c>
       <c r="L5" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>M1.1 — RBAC engine + Resource×Action enum</t>
         </is>
       </c>
     </row>
@@ -2407,7 +2427,12 @@
       </c>
       <c r="L6" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>M1.1 — Permission Matrix UI (Executive only)</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2492,12 @@
       </c>
       <c r="L7" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>M1.1 — Session mgmt + Redis blacklist + broadcast logout</t>
         </is>
       </c>
     </row>
@@ -2527,7 +2557,12 @@
       </c>
       <c r="L8" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>M1.1 — Account lock after failed login attempts</t>
         </is>
       </c>
     </row>
@@ -2587,7 +2622,12 @@
       </c>
       <c r="L9" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>M1.1 — Forgot password + reset via token</t>
         </is>
       </c>
     </row>
@@ -2647,7 +2687,12 @@
       </c>
       <c r="L10" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>M1.1 — Settings page (theme, font, BFA toggle)</t>
         </is>
       </c>
     </row>
@@ -2707,7 +2752,12 @@
       </c>
       <c r="L11" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>M1.1 — Mobile responsive AppShell (Sider + Drawer)</t>
         </is>
       </c>
     </row>
@@ -2767,7 +2817,12 @@
       </c>
       <c r="L12" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>M1.1 — LoginPage UI dengan NIK login</t>
         </is>
       </c>
     </row>
@@ -2827,7 +2882,12 @@
       </c>
       <c r="L13" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>M1.1 — AuditLog model + audit_log() helper, persona name eksplisit</t>
         </is>
       </c>
     </row>
@@ -2887,7 +2947,12 @@
       </c>
       <c r="L14" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>M1.1 — GlobalSearch Cmd+K (Employee + Project)</t>
         </is>
       </c>
     </row>
@@ -2947,7 +3012,12 @@
       </c>
       <c r="L15" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>M1.2 — Employee CRUD + bulk import + filter</t>
         </is>
       </c>
     </row>
@@ -3007,7 +3077,12 @@
       </c>
       <c r="L16" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>M1.2 — EmployeeCreatePage form + EmployeeDetailPage tabs</t>
         </is>
       </c>
     </row>
@@ -3067,7 +3142,12 @@
       </c>
       <c r="L17" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>M1.2 — OrgChartPage tree visualization</t>
         </is>
       </c>
     </row>
@@ -3127,7 +3207,12 @@
       </c>
       <c r="L18" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>M1.2 — Department + Position CRUD</t>
         </is>
       </c>
     </row>
@@ -3187,7 +3272,7 @@
       </c>
       <c r="L19" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3332,12 @@
       </c>
       <c r="L20" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>M1.2 — BPJS fields di Employee + Contract</t>
         </is>
       </c>
     </row>
@@ -3307,7 +3397,12 @@
       </c>
       <c r="L21" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>M1.2 — Employee status lifecycle (PROBATION/ACTIVE/...)</t>
         </is>
       </c>
     </row>
@@ -3367,7 +3462,12 @@
       </c>
       <c r="L22" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>M1.2 — ContractsListPage — PKWT/PKWTT tracking + expiry</t>
         </is>
       </c>
     </row>
@@ -3427,7 +3527,7 @@
       </c>
       <c r="L23" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3487,7 +3587,7 @@
       </c>
       <c r="L24" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3547,7 +3647,7 @@
       </c>
       <c r="L25" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3607,7 +3707,12 @@
       </c>
       <c r="L26" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>M1.2 — OrgChartPage auto-build dari Department + Employee</t>
         </is>
       </c>
     </row>
@@ -3667,7 +3772,12 @@
       </c>
       <c r="L27" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>M1.2 — EmployeeListPage dengan filter + pagination</t>
         </is>
       </c>
     </row>
@@ -3727,7 +3837,12 @@
       </c>
       <c r="L28" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>M1.2 — WorkCalendar + Holiday model</t>
         </is>
       </c>
     </row>
@@ -3787,7 +3902,12 @@
       </c>
       <c r="L29" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>M1.2 — Vendor model + CRUD endpoint (TSK-023)</t>
         </is>
       </c>
     </row>
@@ -3847,7 +3967,12 @@
       </c>
       <c r="L30" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>M1.2 — Client model di Organization domain</t>
         </is>
       </c>
     </row>
@@ -3907,7 +4032,12 @@
       </c>
       <c r="L31" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>M1.3 — JobOpening + JobApplication models + approval flow</t>
         </is>
       </c>
     </row>
@@ -3967,7 +4097,12 @@
       </c>
       <c r="L32" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>M1.3 — JobOpeningCreatePage form</t>
         </is>
       </c>
     </row>
@@ -4027,7 +4162,12 @@
       </c>
       <c r="L33" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>M1.3 — Generic 2-layer approval pattern (leave/reimb/proc/sep/hiring)</t>
         </is>
       </c>
     </row>
@@ -4087,7 +4227,12 @@
       </c>
       <c r="L34" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>M1.3 — Candidate stages: APPLIED → INTERVIEW → OFFERED → HIRED/REJECTED</t>
         </is>
       </c>
     </row>
@@ -4147,7 +4292,12 @@
       </c>
       <c r="L35" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>M1.3 — JobOpening stages config</t>
         </is>
       </c>
     </row>
@@ -4267,7 +4417,12 @@
       </c>
       <c r="L37" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>M1.3 — Candidate status tracking + filter</t>
         </is>
       </c>
     </row>
@@ -4447,7 +4602,12 @@
       </c>
       <c r="L40" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>M1.3 — JobOpeningListPage dashboard</t>
         </is>
       </c>
     </row>
@@ -4507,7 +4667,12 @@
       </c>
       <c r="L41" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>M1.3 — Onboarding template + auto-checklist generation</t>
         </is>
       </c>
     </row>
@@ -4627,7 +4792,12 @@
       </c>
       <c r="L43" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>M1.3 — OnboardingTask items + completion tracking</t>
         </is>
       </c>
     </row>
@@ -5887,7 +6057,12 @@
       </c>
       <c r="L64" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>M2.1 (CLAUDE.md TSK-022) — Project CRUD + members</t>
         </is>
       </c>
     </row>
@@ -5947,7 +6122,12 @@
       </c>
       <c r="L65" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>M2.1 — ProjectMember + allocation_pct</t>
         </is>
       </c>
     </row>
@@ -6007,7 +6187,12 @@
       </c>
       <c r="L66" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>M2.1 (TSK-022 + TSK-022B) — Kanban board, informatif card di TSK-022B</t>
         </is>
       </c>
     </row>
@@ -6127,7 +6312,12 @@
       </c>
       <c r="L68" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>M2.1 — Task CRUD + status + assignee + slug Jira-style</t>
         </is>
       </c>
     </row>
@@ -6187,7 +6377,12 @@
       </c>
       <c r="L69" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>M2.1 → TSK-022B — Milestone replaced by Phase (4-level hierarchy)</t>
         </is>
       </c>
     </row>
@@ -6307,7 +6502,12 @@
       </c>
       <c r="L71" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>M2.1 — Project close flow + Direktur override</t>
         </is>
       </c>
     </row>
@@ -6607,7 +6807,12 @@
       </c>
       <c r="L76" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>M2.1 — Project lifecycle DRAFT/ACTIVE/ON_HOLD/COMPLETED/TERMINATED</t>
         </is>
       </c>
     </row>
@@ -6787,7 +6992,12 @@
       </c>
       <c r="L79" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>M2.1 (CLAUDE.md TSK-021) — OKR objectives + key results</t>
         </is>
       </c>
     </row>
@@ -6847,7 +7057,12 @@
       </c>
       <c r="L80" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>M2.1 — Assessment form per period</t>
         </is>
       </c>
     </row>
@@ -6907,7 +7122,12 @@
       </c>
       <c r="L81" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>M2.1 — Assessment weight config per dept</t>
         </is>
       </c>
     </row>
@@ -6967,7 +7187,12 @@
       </c>
       <c r="L82" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>M2.1 — Score calc (OKR + weighted) → final score</t>
         </is>
       </c>
     </row>
@@ -7027,7 +7252,12 @@
       </c>
       <c r="L83" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>M2.1 — SP threshold flag (kuning→oranye→merah→SP auto)</t>
         </is>
       </c>
     </row>
@@ -7087,7 +7317,12 @@
       </c>
       <c r="L84" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>M2.1 — PerformancePage history tab</t>
         </is>
       </c>
     </row>
@@ -7927,7 +8162,12 @@
       </c>
       <c r="L98" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>M2.2 (TSK-022C+D) — Invoice CRUD di app/finance + UI aging bucket</t>
         </is>
       </c>
     </row>
@@ -7987,7 +8227,12 @@
       </c>
       <c r="L99" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>M2.2 (TSK-022D) — Aging bucket coloring (CURRENT/1-30/31-60/61-90/90+)</t>
         </is>
       </c>
     </row>
@@ -8827,7 +9072,12 @@
       </c>
       <c r="L113" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>M2.3 (CLAUDE.md TSK-019) — Leave request + 2-layer approval</t>
         </is>
       </c>
     </row>
@@ -8887,7 +9137,12 @@
       </c>
       <c r="L114" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>M2.3 — Leave balance engine (annual + sick + maternity)</t>
         </is>
       </c>
     </row>
@@ -8947,7 +9202,12 @@
       </c>
       <c r="L115" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>M2.3 — Leave types (ANNUAL/SICK/MATERNITY/...) config</t>
         </is>
       </c>
     </row>
@@ -9187,7 +9447,12 @@
       </c>
       <c r="L119" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>M2.3 (CLAUDE.md TSK-023) — Reimbursement request + 2-layer approval</t>
         </is>
       </c>
     </row>
@@ -9247,7 +9512,12 @@
       </c>
       <c r="L120" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>M2.3 — Finance reimbursement processing + transfer</t>
         </is>
       </c>
     </row>
@@ -9307,7 +9577,12 @@
       </c>
       <c r="L121" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>M2.3 — Reimbursement history dengan filter</t>
         </is>
       </c>
     </row>
@@ -9427,7 +9702,12 @@
       </c>
       <c r="L123" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>M2.3 — Procurement request + categories</t>
         </is>
       </c>
     </row>
@@ -9487,7 +9767,12 @@
       </c>
       <c r="L124" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>M2.3 — Procurement status tracking + PO + delivery</t>
         </is>
       </c>
     </row>
@@ -9667,7 +9952,12 @@
       </c>
       <c r="L127" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>M3.1 (CLAUDE.md TSK-024) — Lead CRUD + assignee + estimated value</t>
         </is>
       </c>
     </row>
@@ -9727,7 +10017,12 @@
       </c>
       <c r="L128" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>M3.1 — Lead 6-stage funnel (PROSPECT→...→CLOSED_WON/LOST)</t>
         </is>
       </c>
     </row>
@@ -9787,7 +10082,12 @@
       </c>
       <c r="L129" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>M3.1 — Stage transition rules + auto commission di CLOSED_WON</t>
         </is>
       </c>
     </row>
@@ -9847,7 +10147,12 @@
       </c>
       <c r="L130" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>M3.1 — LeadActivity log (call/email/meeting/note)</t>
         </is>
       </c>
     </row>
@@ -13747,7 +14052,7 @@
       </c>
       <c r="L195" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -14228,6 +14533,201 @@
       <c r="L203" t="inlineStr">
         <is>
           <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>TSK-022B</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>EP-07</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Project Management</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>PH2</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>Refactor</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>PM hierarchy Phase&gt;Epic&gt;Task&gt;Subtask + comments</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>Replace Milestone with Phase (4-level), add Epic &amp; Subtask, slug Jira-style + story_points, markdown comments via kanban card</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="I204" t="n">
+        <v>17</v>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>TSK-022C</t>
+        </is>
+      </c>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>Backend+Frontend</t>
+        </is>
+      </c>
+      <c r="L204" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M204" t="inlineStr">
+        <is>
+          <t>M2.1 (refactor) — commit e562724</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>TSK-022C</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>EP-07+EP-09</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Project Management → Finance</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>PH2</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>Refactor</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>Extract Invoice from Project to Finance domain</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>Pindahkan tabel project_invoices ke app/finance/Invoice; trigger source milestone → Phase completion</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="I205" t="n">
+        <v>10</v>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>TSK-022</t>
+        </is>
+      </c>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>Backend+Frontend</t>
+        </is>
+      </c>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M205" t="inlineStr">
+        <is>
+          <t>M2.2 (refactor) — commit 77dbc16</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>TSK-022D</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>EP-09</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Finance Invoice UI</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>PH2</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>Finance Invoice UI — list, create, payment, aging</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>InvoicesTab di FinancePage dengan KPI strip, status filter, aging bucket color, payment tracking modal, PPN auto-compute</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I206" t="n">
+        <v>10</v>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>TSK-022C</t>
+        </is>
+      </c>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M206" t="inlineStr">
+        <is>
+          <t>M2.2 — commit af20538</t>
         </is>
       </c>
     </row>
@@ -24687,8 +25187,8 @@
   <mergeCells count="9">
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A15:L15"/>
+    <mergeCell ref="A52:L52"/>
     <mergeCell ref="A29:L29"/>
-    <mergeCell ref="A52:L52"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A37:L37"/>
     <mergeCell ref="A45:L45"/>

</xml_diff>

<commit_message>
docs: NC-DEV-005/006/007 + mark 20 TSK Done after marathon
CLAUDE.md updates:
- NC-DEV-005: AntD imperative API via @/lib/notify proxy (post audit)
- NC-DEV-006: AntD deprecated props (destroyOnClose, Dropdown overlay)
- NC-DEV-007: WeasyPrint lazy import (avoid startup crash without
  native pango/glib libs)
- Decision Log: 5 new entries 2026-05-31 (notify proxy, sweep,
  audit script, WeasyPrint pattern)

IDEA_Task_Management.xlsx:
- Mark 20 TSK as Done from marathon session (28-31 May):
  TSK-046, 051, 065, 068, 070, 075, 100, 103-109, 148, 150-152, 194, 201
- Backlog progress: 88/204 (43%) — was 68/204 (33%)
</commit_message>
<xml_diff>
--- a/IDEA_Task_Management.xlsx
+++ b/IDEA_Task_Management.xlsx
@@ -373,7 +373,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -576,6 +576,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -5097,7 +5100,7 @@
       </c>
       <c r="L48" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -5397,7 +5400,7 @@
       </c>
       <c r="L53" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6252,7 +6255,7 @@
       </c>
       <c r="L67" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6442,7 +6445,7 @@
       </c>
       <c r="L70" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6567,7 +6570,7 @@
       </c>
       <c r="L72" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6872,7 +6875,7 @@
       </c>
       <c r="L77" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8412,7 +8415,7 @@
       </c>
       <c r="L102" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8592,7 +8595,7 @@
       </c>
       <c r="L105" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8652,7 +8655,7 @@
       </c>
       <c r="L106" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8712,7 +8715,7 @@
       </c>
       <c r="L107" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8772,7 +8775,7 @@
       </c>
       <c r="L108" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8832,7 +8835,7 @@
       </c>
       <c r="L109" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8892,7 +8895,7 @@
       </c>
       <c r="L110" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8952,7 +8955,7 @@
       </c>
       <c r="L111" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -11352,7 +11355,7 @@
       </c>
       <c r="L150" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -11472,7 +11475,7 @@
       </c>
       <c r="L152" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -11532,7 +11535,7 @@
       </c>
       <c r="L153" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -11592,7 +11595,7 @@
       </c>
       <c r="L154" s="37" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -14110,9 +14113,9 @@
           <t>BE+FE</t>
         </is>
       </c>
-      <c r="L196" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="L196" s="74" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -14530,9 +14533,9 @@
           <t>FE</t>
         </is>
       </c>
-      <c r="L203" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="L203" s="74" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -25187,8 +25190,8 @@
   <mergeCells count="9">
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A15:L15"/>
+    <mergeCell ref="A29:L29"/>
     <mergeCell ref="A52:L52"/>
-    <mergeCell ref="A29:L29"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A37:L37"/>
     <mergeCell ref="A45:L45"/>

</xml_diff>

<commit_message>
chore(sprint): formalize Sprint Planning S1-S4 + sprint discipline rule
Sprint Planning sheet (xlsx):
- S1 (1-14 Jun 2026) — M1.4 Payroll core: TSK-047/048/049/050/052/055/056 = 36 pts
- S2 (15-28 Jun 2026) — M1.4 variants + M1.2 UI: TSK-053/054/059/061/197/198/199 = 36 pts
- S3 (29 Jun-12 Jul) — M1.3 closure: TSK-034/036/037/040/042/043/044/045 = 37 pts
- S4 (13-26 Jul) — PH1 GATE Demo + sign-off

Setiap sprint punya goal, dates, task list, status, milestone label.
Total path ke PH1 GATE: 126 pts dalam 4 sprint × 2 minggu = 8 minggu.

CLAUDE.md Decision Log: tambah row 'kembali ke sprint discipline' —
marathon mode bypass roadmap (skip ahead ke PH2 sambil M1.4 baru 37%),
formalkan sprint goals lagi sebelum lanjut.
</commit_message>
<xml_diff>
--- a/IDEA_Task_Management.xlsx
+++ b/IDEA_Task_Management.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="29">
+  <fonts count="35">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -194,8 +194,32 @@
       <strike val="1"/>
       <color rgb="00999999"/>
     </font>
+    <font/>
+    <font>
+      <b val="1"/>
+      <color rgb="001d1d1f"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="006E6E73"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000071E3"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -262,8 +286,20 @@
         <fgColor rgb="0000B0F0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F4FF"/>
+        <bgColor rgb="00F0F4FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000071E3"/>
+        <bgColor rgb="000071E3"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -369,11 +405,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border/>
+    <border>
+      <left style="thin">
+        <color rgb="00D2D2D7"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D2D2D7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D2D2D7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D2D2D7"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -579,6 +630,37 @@
     <xf numFmtId="0" fontId="22" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="14" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="15" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -25190,8 +25272,8 @@
   <mergeCells count="9">
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A15:L15"/>
+    <mergeCell ref="A52:L52"/>
     <mergeCell ref="A29:L29"/>
-    <mergeCell ref="A52:L52"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A37:L37"/>
     <mergeCell ref="A45:L45"/>
@@ -26921,156 +27003,1452 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:I50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
     <col width="6" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="25" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="33" t="inlineStr">
-        <is>
-          <t>SPRINT PLANNING TEMPLATE</t>
-        </is>
-      </c>
+      <c r="A1" s="75" t="inlineStr">
+        <is>
+          <t>SPRINT PLANNING — IDEA Internal Portal</t>
+        </is>
+      </c>
+      <c r="I1" s="76" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="77" t="inlineStr">
+        <is>
+          <t>Kickoff: 1 Jun 2026 · Sprint length: 2 minggu · Velocity target: 30-40 pts (solo+AI)</t>
+        </is>
+      </c>
+      <c r="I2" s="76" t="n"/>
     </row>
     <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="60" t="inlineStr">
-        <is>
-          <t>Sprint #</t>
-        </is>
-      </c>
-      <c r="B3" s="61" t="inlineStr"/>
-      <c r="C3" s="72" t="n"/>
-      <c r="D3" s="73" t="n"/>
+      <c r="A3" s="76" t="n"/>
+      <c r="B3" s="76" t="n"/>
+      <c r="C3" s="76" t="n"/>
+      <c r="D3" s="76" t="n"/>
+      <c r="E3" s="76" t="n"/>
+      <c r="F3" s="76" t="n"/>
+      <c r="G3" s="76" t="n"/>
+      <c r="H3" s="76" t="n"/>
+      <c r="I3" s="76" t="n"/>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="60" t="inlineStr">
-        <is>
-          <t>Sprint Goal</t>
-        </is>
-      </c>
-      <c r="B4" s="61" t="inlineStr"/>
-      <c r="C4" s="72" t="n"/>
-      <c r="D4" s="73" t="n"/>
+      <c r="A4" s="78" t="inlineStr">
+        <is>
+          <t>SPRINT 1  ·  1 – 14 Jun 2026</t>
+        </is>
+      </c>
+      <c r="I4" s="76" t="n"/>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="60" t="inlineStr">
-        <is>
-          <t>Start Date</t>
-        </is>
-      </c>
-      <c r="B5" s="61" t="inlineStr"/>
-      <c r="C5" s="72" t="n"/>
-      <c r="D5" s="73" t="n"/>
+      <c r="A5" s="77" t="inlineStr">
+        <is>
+          <t>🎯 Goal: Payroll engine end-to-end: attendance → calc → review → slip</t>
+        </is>
+      </c>
+      <c r="I5" s="76" t="n"/>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="60" t="inlineStr">
-        <is>
-          <t>End Date</t>
-        </is>
-      </c>
-      <c r="B6" s="61" t="inlineStr"/>
-      <c r="C6" s="72" t="n"/>
-      <c r="D6" s="73" t="n"/>
+      <c r="A6" s="79" t="inlineStr">
+        <is>
+          <t>Task ID</t>
+        </is>
+      </c>
+      <c r="B6" s="79" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="C6" s="79" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="D6" s="79" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E6" s="79" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="F6" s="79" t="inlineStr">
+        <is>
+          <t>Pts</t>
+        </is>
+      </c>
+      <c r="G6" s="79" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H6" s="79" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="I6" s="76" t="n"/>
     </row>
     <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="60" t="inlineStr">
-        <is>
-          <t>Team Capacity (hrs)</t>
-        </is>
-      </c>
-      <c r="B7" s="61" t="inlineStr"/>
-      <c r="C7" s="72" t="n"/>
-      <c r="D7" s="73" t="n"/>
+      <c r="A7" s="80" t="inlineStr">
+        <is>
+          <t>TSK-047</t>
+        </is>
+      </c>
+      <c r="B7" s="80" t="inlineStr">
+        <is>
+          <t>EP-05</t>
+        </is>
+      </c>
+      <c r="C7" s="80" t="inlineStr">
+        <is>
+          <t>Monthly Attendance Input by Operation</t>
+        </is>
+      </c>
+      <c r="D7" s="81" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="E7" s="81" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F7" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="G7" s="81" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H7" s="81" t="inlineStr">
+        <is>
+          <t>M1.4</t>
+        </is>
+      </c>
+      <c r="I7" s="76" t="n"/>
     </row>
     <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="60" t="inlineStr">
-        <is>
-          <t>Sprint Velocity</t>
-        </is>
-      </c>
-      <c r="B8" s="61" t="inlineStr"/>
-      <c r="C8" s="72" t="n"/>
-      <c r="D8" s="73" t="n"/>
-    </row>
-    <row r="10" ht="12" customHeight="1"/>
+      <c r="A8" s="80" t="inlineStr">
+        <is>
+          <t>TSK-048</t>
+        </is>
+      </c>
+      <c r="B8" s="80" t="inlineStr">
+        <is>
+          <t>EP-05</t>
+        </is>
+      </c>
+      <c r="C8" s="80" t="inlineStr">
+        <is>
+          <t>Payroll Calculation Engine</t>
+        </is>
+      </c>
+      <c r="D8" s="81" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="E8" s="81" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F8" s="81" t="n">
+        <v>13</v>
+      </c>
+      <c r="G8" s="81" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H8" s="81" t="inlineStr">
+        <is>
+          <t>M1.4</t>
+        </is>
+      </c>
+      <c r="I8" s="76" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="80" t="inlineStr">
+        <is>
+          <t>TSK-049</t>
+        </is>
+      </c>
+      <c r="B9" s="80" t="inlineStr">
+        <is>
+          <t>EP-05</t>
+        </is>
+      </c>
+      <c r="C9" s="80" t="inlineStr">
+        <is>
+          <t>PPh 21 Manual Input per Employee</t>
+        </is>
+      </c>
+      <c r="D9" s="81" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="E9" s="81" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F9" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="G9" s="81" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H9" s="81" t="inlineStr">
+        <is>
+          <t>M1.4</t>
+        </is>
+      </c>
+      <c r="I9" s="76" t="n"/>
+    </row>
+    <row r="10" ht="12" customHeight="1">
+      <c r="A10" s="80" t="inlineStr">
+        <is>
+          <t>TSK-050</t>
+        </is>
+      </c>
+      <c r="B10" s="80" t="inlineStr">
+        <is>
+          <t>EP-05</t>
+        </is>
+      </c>
+      <c r="C10" s="80" t="inlineStr">
+        <is>
+          <t>Payroll Review &amp; Approval by GM/CLevel</t>
+        </is>
+      </c>
+      <c r="D10" s="81" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="E10" s="81" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F10" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="G10" s="81" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H10" s="81" t="inlineStr">
+        <is>
+          <t>M1.4</t>
+        </is>
+      </c>
+      <c r="I10" s="76" t="n"/>
+    </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="80" t="inlineStr">
+        <is>
+          <t>TSK-052</t>
+        </is>
+      </c>
+      <c r="B11" s="80" t="inlineStr">
+        <is>
+          <t>EP-05</t>
+        </is>
+      </c>
+      <c r="C11" s="80" t="inlineStr">
+        <is>
+          <t>Pay Slip History Access</t>
+        </is>
+      </c>
+      <c r="D11" s="81" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="E11" s="81" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F11" s="81" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" s="81" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H11" s="81" t="inlineStr">
+        <is>
+          <t>M1.4</t>
+        </is>
+      </c>
+      <c r="I11" s="76" t="n"/>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="80" t="inlineStr">
+        <is>
+          <t>TSK-055</t>
+        </is>
+      </c>
+      <c r="B12" s="80" t="inlineStr">
+        <is>
+          <t>EP-05</t>
+        </is>
+      </c>
+      <c r="C12" s="80" t="inlineStr">
+        <is>
+          <t>Payroll Period Configuration</t>
+        </is>
+      </c>
+      <c r="D12" s="81" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="E12" s="81" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F12" s="81" t="n">
+        <v>3</v>
+      </c>
+      <c r="G12" s="81" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H12" s="81" t="inlineStr">
+        <is>
+          <t>M1.4</t>
+        </is>
+      </c>
+      <c r="I12" s="76" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="82" t="inlineStr">
+        <is>
+          <t>TSK-056</t>
+        </is>
+      </c>
+      <c r="B13" s="82" t="inlineStr">
+        <is>
+          <t>EP-05</t>
+        </is>
+      </c>
+      <c r="C13" s="82" t="inlineStr">
+        <is>
+          <t>Payroll Duplicate Prevention</t>
+        </is>
+      </c>
+      <c r="D13" s="83" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="E13" s="83" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F13" s="83" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" s="83" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H13" s="83" t="inlineStr">
+        <is>
+          <t>M1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="E14" s="84" t="inlineStr">
+        <is>
+          <t>TOTAL:</t>
+        </is>
+      </c>
+      <c r="F14" s="85" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="86" t="inlineStr">
+        <is>
+          <t>SPRINT 2  ·  15 – 28 Jun 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="87" t="inlineStr">
+        <is>
+          <t>🎯 Goal: M1.4 payroll variants (THR, prorated) + Alert Rules + M1.2 UI closure</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="79" t="inlineStr">
         <is>
           <t>Task ID</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B18" s="79" t="inlineStr">
         <is>
           <t>Epic</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C18" s="79" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D18" s="79" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E18" s="79" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F18" s="79" t="inlineStr">
         <is>
           <t>Pts</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>Assignee</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="G18" s="79" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="62" t="inlineStr">
-        <is>
-          <t>TOTAL STORY POINTS (Phase 1 Critical/High suggestion)</t>
-        </is>
-      </c>
-      <c r="F12" s="63">
-        <f>SUM(F12:F11)</f>
-        <v/>
+      <c r="H18" s="79" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="82" t="inlineStr">
+        <is>
+          <t>TSK-053</t>
+        </is>
+      </c>
+      <c r="B19" s="82" t="inlineStr">
+        <is>
+          <t>EP-05</t>
+        </is>
+      </c>
+      <c r="C19" s="82" t="inlineStr">
+        <is>
+          <t>THR Processing Module</t>
+        </is>
+      </c>
+      <c r="D19" s="83" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="E19" s="83" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F19" s="83" t="n">
+        <v>5</v>
+      </c>
+      <c r="G19" s="83" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H19" s="83" t="inlineStr">
+        <is>
+          <t>M1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="82" t="inlineStr">
+        <is>
+          <t>TSK-054</t>
+        </is>
+      </c>
+      <c r="B20" s="82" t="inlineStr">
+        <is>
+          <t>EP-05</t>
+        </is>
+      </c>
+      <c r="C20" s="82" t="inlineStr">
+        <is>
+          <t>Prorated Final Payroll (Exit)</t>
+        </is>
+      </c>
+      <c r="D20" s="83" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="E20" s="83" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F20" s="83" t="n">
+        <v>5</v>
+      </c>
+      <c r="G20" s="83" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H20" s="83" t="inlineStr">
+        <is>
+          <t>M1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="82" t="inlineStr">
+        <is>
+          <t>TSK-059</t>
+        </is>
+      </c>
+      <c r="B21" s="82" t="inlineStr">
+        <is>
+          <t>EP-06</t>
+        </is>
+      </c>
+      <c r="C21" s="82" t="inlineStr">
+        <is>
+          <t>Alert Rules Engine</t>
+        </is>
+      </c>
+      <c r="D21" s="83" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="E21" s="83" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F21" s="83" t="n">
+        <v>8</v>
+      </c>
+      <c r="G21" s="83" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H21" s="83" t="inlineStr">
+        <is>
+          <t>M1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="82" t="inlineStr">
+        <is>
+          <t>TSK-061</t>
+        </is>
+      </c>
+      <c r="B22" s="82" t="inlineStr">
+        <is>
+          <t>EP-06</t>
+        </is>
+      </c>
+      <c r="C22" s="82" t="inlineStr">
+        <is>
+          <t>Notification Retry &amp; Failure Handling</t>
+        </is>
+      </c>
+      <c r="D22" s="83" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="E22" s="83" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F22" s="83" t="n">
+        <v>3</v>
+      </c>
+      <c r="G22" s="83" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H22" s="83" t="inlineStr">
+        <is>
+          <t>M1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="82" t="inlineStr">
+        <is>
+          <t>TSK-197</t>
+        </is>
+      </c>
+      <c r="B23" s="82" t="inlineStr">
+        <is>
+          <t>EP-02</t>
+        </is>
+      </c>
+      <c r="C23" s="82" t="inlineStr">
+        <is>
+          <t>Promotion UI Page (US-OP-012)</t>
+        </is>
+      </c>
+      <c r="D23" s="83" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="E23" s="83" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F23" s="83" t="n">
+        <v>5</v>
+      </c>
+      <c r="G23" s="83" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H23" s="83" t="inlineStr">
+        <is>
+          <t>M1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="82" t="inlineStr">
+        <is>
+          <t>TSK-198</t>
+        </is>
+      </c>
+      <c r="B24" s="82" t="inlineStr">
+        <is>
+          <t>EP-02</t>
+        </is>
+      </c>
+      <c r="C24" s="82" t="inlineStr">
+        <is>
+          <t>Mutation UI Page (US-OP-013)</t>
+        </is>
+      </c>
+      <c r="D24" s="83" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="E24" s="83" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F24" s="83" t="n">
+        <v>5</v>
+      </c>
+      <c r="G24" s="83" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H24" s="83" t="inlineStr">
+        <is>
+          <t>M1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="82" t="inlineStr">
+        <is>
+          <t>TSK-199</t>
+        </is>
+      </c>
+      <c r="B25" s="82" t="inlineStr">
+        <is>
+          <t>EP-02</t>
+        </is>
+      </c>
+      <c r="C25" s="82" t="inlineStr">
+        <is>
+          <t>PKWT Renewal Decision UI (US-OP-014)</t>
+        </is>
+      </c>
+      <c r="D25" s="83" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="E25" s="83" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F25" s="83" t="n">
+        <v>5</v>
+      </c>
+      <c r="G25" s="83" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H25" s="83" t="inlineStr">
+        <is>
+          <t>M1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="E26" s="84" t="inlineStr">
+        <is>
+          <t>TOTAL:</t>
+        </is>
+      </c>
+      <c r="F26" s="85" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="86" t="inlineStr">
+        <is>
+          <t>SPRINT 3  ·  29 Jun – 12 Jul 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="87" t="inlineStr">
+        <is>
+          <t>🎯 Goal: M1.3 closure: hiring + onboarding (probation, welcome, CMS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="79" t="inlineStr">
+        <is>
+          <t>Task ID</t>
+        </is>
+      </c>
+      <c r="B30" s="79" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="C30" s="79" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="D30" s="79" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E30" s="79" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="F30" s="79" t="inlineStr">
+        <is>
+          <t>Pts</t>
+        </is>
+      </c>
+      <c r="G30" s="79" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H30" s="79" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="82" t="inlineStr">
+        <is>
+          <t>TSK-034</t>
+        </is>
+      </c>
+      <c r="B31" s="82" t="inlineStr">
+        <is>
+          <t>EP-03</t>
+        </is>
+      </c>
+      <c r="C31" s="82" t="inlineStr">
+        <is>
+          <t>Offering Letter Generation</t>
+        </is>
+      </c>
+      <c r="D31" s="83" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="E31" s="83" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F31" s="83" t="n">
+        <v>8</v>
+      </c>
+      <c r="G31" s="83" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H31" s="83" t="inlineStr">
+        <is>
+          <t>M1.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="82" t="inlineStr">
+        <is>
+          <t>TSK-036</t>
+        </is>
+      </c>
+      <c r="B32" s="82" t="inlineStr">
+        <is>
+          <t>EP-03</t>
+        </is>
+      </c>
+      <c r="C32" s="82" t="inlineStr">
+        <is>
+          <t>Internal Job Board</t>
+        </is>
+      </c>
+      <c r="D32" s="83" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="E32" s="83" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F32" s="83" t="n">
+        <v>3</v>
+      </c>
+      <c r="G32" s="83" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H32" s="83" t="inlineStr">
+        <is>
+          <t>M1.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="82" t="inlineStr">
+        <is>
+          <t>TSK-037</t>
+        </is>
+      </c>
+      <c r="B33" s="82" t="inlineStr">
+        <is>
+          <t>EP-03</t>
+        </is>
+      </c>
+      <c r="C33" s="82" t="inlineStr">
+        <is>
+          <t>Duplicate Request Detection</t>
+        </is>
+      </c>
+      <c r="D33" s="83" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="E33" s="83" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F33" s="83" t="n">
+        <v>2</v>
+      </c>
+      <c r="G33" s="83" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H33" s="83" t="inlineStr">
+        <is>
+          <t>M1.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="82" t="inlineStr">
+        <is>
+          <t>TSK-040</t>
+        </is>
+      </c>
+      <c r="B34" s="82" t="inlineStr">
+        <is>
+          <t>EP-04</t>
+        </is>
+      </c>
+      <c r="C34" s="82" t="inlineStr">
+        <is>
+          <t>Welcome Page for New Employees</t>
+        </is>
+      </c>
+      <c r="D34" s="83" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="E34" s="83" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F34" s="83" t="n">
+        <v>5</v>
+      </c>
+      <c r="G34" s="83" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H34" s="83" t="inlineStr">
+        <is>
+          <t>M1.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="82" t="inlineStr">
+        <is>
+          <t>TSK-042</t>
+        </is>
+      </c>
+      <c r="B35" s="82" t="inlineStr">
+        <is>
+          <t>EP-04</t>
+        </is>
+      </c>
+      <c r="C35" s="82" t="inlineStr">
+        <is>
+          <t>H-3 Pre-join Preparation Alert</t>
+        </is>
+      </c>
+      <c r="D35" s="83" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="E35" s="83" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F35" s="83" t="n">
+        <v>3</v>
+      </c>
+      <c r="G35" s="83" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H35" s="83" t="inlineStr">
+        <is>
+          <t>M1.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="82" t="inlineStr">
+        <is>
+          <t>TSK-043</t>
+        </is>
+      </c>
+      <c r="B36" s="82" t="inlineStr">
+        <is>
+          <t>EP-04</t>
+        </is>
+      </c>
+      <c r="C36" s="82" t="inlineStr">
+        <is>
+          <t>Account Activation on Join Date</t>
+        </is>
+      </c>
+      <c r="D36" s="83" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="E36" s="83" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F36" s="83" t="n">
+        <v>3</v>
+      </c>
+      <c r="G36" s="83" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H36" s="83" t="inlineStr">
+        <is>
+          <t>M1.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="82" t="inlineStr">
+        <is>
+          <t>TSK-044</t>
+        </is>
+      </c>
+      <c r="B37" s="82" t="inlineStr">
+        <is>
+          <t>EP-04</t>
+        </is>
+      </c>
+      <c r="C37" s="82" t="inlineStr">
+        <is>
+          <t>Probation Assessment Flow</t>
+        </is>
+      </c>
+      <c r="D37" s="83" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="E37" s="83" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F37" s="83" t="n">
+        <v>8</v>
+      </c>
+      <c r="G37" s="83" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H37" s="83" t="inlineStr">
+        <is>
+          <t>M1.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="82" t="inlineStr">
+        <is>
+          <t>TSK-045</t>
+        </is>
+      </c>
+      <c r="B38" s="82" t="inlineStr">
+        <is>
+          <t>EP-04</t>
+        </is>
+      </c>
+      <c r="C38" s="82" t="inlineStr">
+        <is>
+          <t>Company Info Portal (CMS)</t>
+        </is>
+      </c>
+      <c r="D38" s="83" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="E38" s="83" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F38" s="83" t="n">
+        <v>5</v>
+      </c>
+      <c r="G38" s="83" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H38" s="83" t="inlineStr">
+        <is>
+          <t>M1.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="E39" s="84" t="inlineStr">
+        <is>
+          <t>TOTAL:</t>
+        </is>
+      </c>
+      <c r="F39" s="85" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="86" t="inlineStr">
+        <is>
+          <t>SPRINT 4  ·  13 – 26 Jul 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="87" t="inlineStr">
+        <is>
+          <t>🎯 Goal: PH1 GATE Demo + sign-off — gerbang ke PH2</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="79" t="inlineStr">
+        <is>
+          <t>Task ID</t>
+        </is>
+      </c>
+      <c r="B43" s="79" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="C43" s="79" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="D43" s="79" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E43" s="79" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="F43" s="79" t="inlineStr">
+        <is>
+          <t>Pts</t>
+        </is>
+      </c>
+      <c r="G43" s="79" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H43" s="79" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="82" t="inlineStr">
+        <is>
+          <t>demo-1</t>
+        </is>
+      </c>
+      <c r="B44" s="82" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C44" s="82" t="inlineStr">
+        <is>
+          <t>Seed 10 dummy karyawan + 1 dept Teknologi full</t>
+        </is>
+      </c>
+      <c r="D44" s="83" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="E44" s="83" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F44" s="83" t="n">
+        <v>2</v>
+      </c>
+      <c r="G44" s="83" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H44" s="83" t="inlineStr">
+        <is>
+          <t>PH1 GATE</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="82" t="inlineStr">
+        <is>
+          <t>demo-2</t>
+        </is>
+      </c>
+      <c r="B45" s="82" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C45" s="82" t="inlineStr">
+        <is>
+          <t>End-to-end smoke test: login → hiring → onboarding → payroll</t>
+        </is>
+      </c>
+      <c r="D45" s="83" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="E45" s="83" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F45" s="83" t="n">
+        <v>3</v>
+      </c>
+      <c r="G45" s="83" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H45" s="83" t="inlineStr">
+        <is>
+          <t>PH1 GATE</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="82" t="inlineStr">
+        <is>
+          <t>demo-3</t>
+        </is>
+      </c>
+      <c r="B46" s="82" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C46" s="82" t="inlineStr">
+        <is>
+          <t>Bug-fix sweep (audit_frontend + audit_models + smoke run)</t>
+        </is>
+      </c>
+      <c r="D46" s="83" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="E46" s="83" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F46" s="83" t="n">
+        <v>5</v>
+      </c>
+      <c r="G46" s="83" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H46" s="83" t="inlineStr">
+        <is>
+          <t>PH1 GATE</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="82" t="inlineStr">
+        <is>
+          <t>demo-4</t>
+        </is>
+      </c>
+      <c r="B47" s="82" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C47" s="82" t="inlineStr">
+        <is>
+          <t>PH1 GATE acceptance checklist (8 kriteria)</t>
+        </is>
+      </c>
+      <c r="D47" s="83" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="E47" s="83" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F47" s="83" t="n">
+        <v>3</v>
+      </c>
+      <c r="G47" s="83" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H47" s="83" t="inlineStr">
+        <is>
+          <t>PH1 GATE</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="82" t="inlineStr">
+        <is>
+          <t>demo-5</t>
+        </is>
+      </c>
+      <c r="B48" s="82" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C48" s="82" t="inlineStr">
+        <is>
+          <t>Stakeholder sign-off prep: Dirut, GM Op, CTO</t>
+        </is>
+      </c>
+      <c r="D48" s="83" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="E48" s="83" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F48" s="83" t="n">
+        <v>2</v>
+      </c>
+      <c r="G48" s="83" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H48" s="83" t="inlineStr">
+        <is>
+          <t>PH1 GATE</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="82" t="inlineStr">
+        <is>
+          <t>demo-6</t>
+        </is>
+      </c>
+      <c r="B49" s="82" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C49" s="82" t="inlineStr">
+        <is>
+          <t>PH2 M2.1 sprint planning + backlog refinement</t>
+        </is>
+      </c>
+      <c r="D49" s="83" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="E49" s="83" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F49" s="83" t="n">
+        <v>2</v>
+      </c>
+      <c r="G49" s="83" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H49" s="83" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="E50" s="84" t="inlineStr">
+        <is>
+          <t>TOTAL:</t>
+        </is>
+      </c>
+      <c r="F50" s="85" t="n">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="A12:E12"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B6:D6"/>
+  <mergeCells count="10">
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A42:H42"/>
+    <mergeCell ref="A41:H41"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A17:H17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>